<commit_message>
Update test-cases.xlsx with all screen tests through phase 5
Extends the 19 phase-3 cases with 27 more covering everything tested
since: maturity matrix and spider chart rendering (both frameworks),
the spider-chart label clipping bug and fix, the Initial-column
removal, the per-checkpoint memo textarea (sizing, wrapping,
persistence), the restored/renamed key-area percentage table, the
"回答をクリアする" confirm modal (including the hidden-attribute
override bug and fix), and the rule-based 短評 feature (all TPI NEXT
stage branches, tie handling, Agile TPI branches, the priority-item
format change, and the edit-preservation-vs-regeneration logic
including the reference-vs-copy bug and fix). 46 cases total.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases.xlsx
+++ b/docs/test-cases.xlsx
@@ -10,7 +10,7 @@
     <sheet name="テストケース" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'テストケース'!$A$1:$J$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'テストケース'!$A$1:$J$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,12 @@
       <color rgb="002E7D5B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Yu Gothic"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -58,7 +64,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -80,11 +86,25 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="medium">
+        <color rgb="001F4478"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,6 +119,21 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -466,19 +501,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -533,7 +568,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>TC-01</t>
@@ -582,7 +617,7 @@
       </c>
       <c r="J2" s="4" t="inlineStr"/>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>TC-02</t>
@@ -635,7 +670,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>TC-03</t>
@@ -688,7 +723,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>TC-04</t>
@@ -741,7 +776,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>TC-05</t>
@@ -790,7 +825,7 @@
       </c>
       <c r="J6" s="4" t="inlineStr"/>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>TC-06</t>
@@ -843,7 +878,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>TC-07</t>
@@ -892,7 +927,7 @@
       </c>
       <c r="J8" s="4" t="inlineStr"/>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>TC-08</t>
@@ -941,7 +976,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr"/>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>TC-09</t>
@@ -978,7 +1013,7 @@
           <t>本文の直下に3択の選択肢が隙間なく表示される</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>PASS（修正前はFAIL）</t>
         </is>
@@ -994,7 +1029,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="72" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>TC-10</t>
@@ -1043,7 +1078,7 @@
       </c>
       <c r="J11" s="4" t="inlineStr"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="72" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>TC-11</t>
@@ -1093,7 +1128,7 @@
       </c>
       <c r="J12" s="4" t="inlineStr"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="72" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>TC-12</t>
@@ -1142,7 +1177,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr"/>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="72" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>TC-13</t>
@@ -1191,7 +1226,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="72" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>TC-14</t>
@@ -1240,7 +1275,7 @@
       </c>
       <c r="J15" s="4" t="inlineStr"/>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="72" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>TC-15</t>
@@ -1290,7 +1325,7 @@
       </c>
       <c r="J16" s="4" t="inlineStr"/>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="72" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>TC-16</t>
@@ -1339,7 +1374,7 @@
       </c>
       <c r="J17" s="4" t="inlineStr"/>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="72" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>TC-17</t>
@@ -1392,7 +1427,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="60" customHeight="1">
+    <row r="19" ht="72" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>TC-18</t>
@@ -1441,7 +1476,7 @@
       </c>
       <c r="J19" s="4" t="inlineStr"/>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20" ht="72" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>TC-19</t>
@@ -1454,7 +1489,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>JSランタイムエラーの非発生確認</t>
+          <t>JSランタイムエラーの非発生確認（フェーズ3）</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -1493,8 +1528,1384 @@
         </is>
       </c>
     </row>
+    <row r="21" ht="72" customHeight="1">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>TC-20</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>成熟度マトリクス</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>TPI NEXT成熟度マトリクスの表示確認</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>キーエリア×段階（Controlled/Efficient/Optimizing）のグリッドに、チェックポイントの回答に応じてセルが緑/赤/グレーで色分けされ、クラスタ文字が表示されること</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>TPI NEXT</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>1. 全157件に回答する
+2. 結果画面のマトリクスセクションを確認する</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>元Excelのマトリクス表と同様の見た目で、各セルに正しい色とクラスタ文字が表示される</t>
+        </is>
+      </c>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I21" s="7" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>列幅は全キーエリア中の最大チェックポイント数に揃えてグリッド状に整列するよう実装</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="72" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>TC-21</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>成熟度マトリクス</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Agile TPI成熟度マトリクスの表示確認</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>キーエリア×3軸（Professional/Team/Organization）のグリッドで同様に色分け表示されること</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Agile TPI</t>
+        </is>
+      </c>
+      <c r="F22" s="4" t="inlineStr">
+        <is>
+          <t>1. 全108件に回答する
+2. 結果画面のマトリクスセクションを確認する</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>3軸の列で正しく色分け・クラスタ文字表示される</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J22" s="4" t="inlineStr"/>
+    </row>
+    <row r="23" ht="72" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>TC-22</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>スパイダーグラフ</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>スパイダーグラフの表示確認</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>16キーエリアを軸としたSVGレーダーチャートが表示され、現在の達成率（実線）と満点ライン（破線）が重ねて表示されること</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F23" s="4" t="inlineStr">
+        <is>
+          <t>1. 結果画面のスパイダーグラフセクションを確認する</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>16軸すべてのラベル・目盛り・2本のポリゴンが表示される</t>
+        </is>
+      </c>
+      <c r="H23" s="6" t="inlineStr">
+        <is>
+          <t>PASS（修正前は軸ラベル見切れでFAIL）</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J23" s="4" t="inlineStr">
+        <is>
+          <t>初期実装でラベルがSVG左右端で見切れる不具合を発見。viewBoxの余白拡大とラベル折返し文字数の調整（8文字→6文字）で修正</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="72" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TC-23</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>レスポンシブ</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>モバイル幅でのマトリクス横スクロール確認</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>マトリクス表がモバイル幅で画面からはみ出る場合、横スクロールで閲覧できること</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>1. モバイル幅（375x812）で結果画面を開く
+2. マトリクスを横スクロールする</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>スクロールコンテナ内でマトリクス全体を横方向に閲覧できる</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr"/>
+    </row>
+    <row r="25" ht="72" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TC-24</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>成熟度マトリクス</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT／Initial列の削除確認</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>チェックポイントを持たないInitial列を非表示にし、Controlled/Efficient/Optimizingの3段階のみ表示されること</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>1. 結果画面のマトリクスヘッダーを確認する</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>Initial列が表示されず、3段階のみのヘッダーになる</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J25" s="4" t="inlineStr">
+        <is>
+          <t>Agile TPI側（軸構成）には影響がないことも確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="72" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TC-25</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>結果画面</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>達成率一覧テーブルの表示確認</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>マトリクス・スパイダーグラフに加えて、キーエリアごとの達成率を一覧表示するテーブルが表示されること</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>1. 結果画面の該当セクションを確認する</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>No./キーエリア/達成率の3列でキーエリア16件分が表示される</t>
+        </is>
+      </c>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>当初「診断結果（簡易表示）」というタイトルで実装し、後に「キーエリア毎の達成率」に改称</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="72" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TC-26</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>メモ機能</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>チェックポイントごとのメモ欄表示確認</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>各チェックポイントの「該当なし」の右側に、メモ入力用テキストエリアが表示されること</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>1. 診断画面を開く
+2. チェックポイント行を確認する</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>プレースホルダー「メモ（任意）」付きのテキストエリアが表示される</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr"/>
+    </row>
+    <row r="28" ht="72" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TC-27</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>メモ機能</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>メモ欄の折り返し・スクロール確認</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>1行あたり全角20文字程度で折り返し、5行分の高さで固定表示され、それを超える入力は縦スクロールで表示されること（自動リサイズしない）</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>1. 20文字・21文字・8行分のテキストを入力する
+2. 折り返しとスクロール発生を確認する</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>20〜21文字は1行に収まり、5行を超える内容はボックス高さを変えずにスクロールする</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>当初15文字幅で実装後、20文字幅に変更。幅は210px→280pxに調整</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="72" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TC-28</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>メモ機能</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>メモ内容のlocalStorage永続化確認</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>メモに入力した内容がlocalStorageに保存され、ページリロード後も復元されること</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>1. メモに入力する
+2. ページを完全リロードする
+3. 内容を確認する</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>リロード後も入力内容が保持されている</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>回答と同じ永続化パターン（tpiAssessmentTool.notes.v1）を使用</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="72" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TC-29</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>レスポンシブ</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>モバイル幅でのメモ欄配置確認</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>モバイル幅ではラジオボタンとメモ欄が折り返して縦に並ぶこと</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>1. モバイル幅で診断画面のチェックポイント行を確認する</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>選択肢・メモ欄が適切に折り返され、崩れがない</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr"/>
+    </row>
+    <row r="31" ht="72" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TC-30</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>回答クリア機能</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>ボタン・確認モーダルの表示確認</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>診断画面上部の「回答をクリアする」ボタン押下で、確認メッセージと「キャンセル」「削除する」ボタンを持つモーダルが表示されること</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>1. 診断画面で「回答をクリアする」を押す</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>モーダルが表示され、背景がオーバーレイで暗くなる</t>
+        </is>
+      </c>
+      <c r="H31" s="6" t="inlineStr">
+        <is>
+          <t>PASS（修正前はモーダル常時表示でFAIL）</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>`.modal-overlay`のdisplay:flexがhidden属性のデフォルト非表示を上書きしてしまう不具合を発見・修正（`.modal-overlay[hidden]{display:none}`を追加）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="72" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TC-31</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>回答クリア機能</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>キャンセル動作確認</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>「キャンセル」押下でモーダルが閉じ、回答内容は変更されないこと</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>1. モーダルを開く
+2. 「キャンセル」を押す</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>モーダルが閉じ、回答は元のまま</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr"/>
+    </row>
+    <row r="33" ht="72" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TC-32</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>回答クリア機能</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>Escapeキー・背景クリックでの挙動確認</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>Escapeキー押下、またはオーバーレイ背景のクリックでモーダルが閉じること。ダイアログ内のクリックでは閉じないこと</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>1. モーダルを開いた状態でEscapeキーを送出する
+2. 背景をクリックする
+3. ダイアログ内タイトルをクリックする</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>Escapeと背景クリックでは閉じる。ダイアログ内クリックでは閉じない</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr"/>
+    </row>
+    <row r="34" ht="72" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TC-33</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>回答クリア機能</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>削除実行時の全項目リセット確認</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>「削除する」押下で、回答・メモがすべて削除され、進捗表示が0件に戻ること</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>1. 全項目回答・メモ入力する
+2. 「回答をクリアする」→「削除する」を実行する</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>進捗が0/157（Agile TPIは0/108）になり、ラジオボタン・メモ欄が空になる</t>
+        </is>
+      </c>
+      <c r="H34" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr"/>
+    </row>
+    <row r="35" ht="72" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>TC-34</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>回答クリア機能</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>フレームワーク間の独立性確認</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>TPI NEXT側で「回答をクリアする」を実行しても、Agile TPI側の下書きには影響しないこと</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F35" s="4" t="inlineStr">
+        <is>
+          <t>1. 両フレームワークに回答する
+2. 片方をクリアする
+3. もう片方のlocalStorageを確認する</t>
+        </is>
+      </c>
+      <c r="G35" s="4" t="inlineStr">
+        <is>
+          <t>クリアしていない側のデータは変化しない</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J35" s="4" t="inlineStr"/>
+    </row>
+    <row r="36" ht="72" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>TC-35</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT／CONTROLLED未達成メッセージ確認</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>CONTROLLEDステージに「満たしていない」チェックポイントがある場合、専用の導入メッセージと優先チェックポイントリストが出力されること</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT</t>
+        </is>
+      </c>
+      <c r="F36" s="4" t="inlineStr">
+        <is>
+          <t>1. CONTROLLEDステージの全チェックポイントを「満たしていない」にする
+2. 結果画面を開く</t>
+        </is>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>「TPI NEXTにおいて、先ずはCONTROLLEDを完全達成を目指すことがセオリーです。」で始まるメッセージと優先リストが表示される</t>
+        </is>
+      </c>
+      <c r="H36" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>同率5位が多数存在するケース（12件表示）でのタイ処理も確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="72" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>TC-36</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT／EFFICIENT未達成メッセージ確認</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>CONTROLLED達成・EFFICIENTに未達成がある場合の専用メッセージ確認</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT</t>
+        </is>
+      </c>
+      <c r="F37" s="4" t="inlineStr">
+        <is>
+          <t>1. CONTROLLEDを全達成、EFFICIENTステージを「満たしていない」にする
+2. 結果画面を開く</t>
+        </is>
+      </c>
+      <c r="G37" s="4" t="inlineStr">
+        <is>
+          <t>「多くの組織において目指すべき目標とされるCONTROLLEDを達成しています。」で始まるメッセージが表示される</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J37" s="4" t="inlineStr"/>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>TC-37</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT／OPTIMIZING未達成メッセージ確認</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>CONTROLLED・EFFICIENT達成、OPTIMIZINGのみ未達成の場合の専用メッセージ確認</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>1. CONTROLLED・EFFICIENTを全達成、OPTIMIZINGステージを「満たしていない」にする
+2. 結果画面を開く</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>「EFFICIENTレベルを達成しており、業界上位の水準での品質組織となっています。」で始まるメッセージが表示される</t>
+        </is>
+      </c>
+      <c r="H38" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr"/>
+    </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>TC-38</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT／全達成メッセージ確認</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>全チェックポイントが「満たしている」または「該当なし」の場合、固定の称賛メッセージのみが表示されること</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>TPI NEXT</t>
+        </is>
+      </c>
+      <c r="F39" s="4" t="inlineStr">
+        <is>
+          <t>1. 全項目を「満たしている」にする
+2. 結果画面を開く</t>
+        </is>
+      </c>
+      <c r="G39" s="4" t="inlineStr">
+        <is>
+          <t>「本プロジェクトの成熟度は業界最高水準に達しています！Excellent！！」が表示される</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J39" s="4" t="inlineStr"/>
+    </row>
+    <row r="40" ht="72" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>TC-39</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Agile TPI優先リスト確認</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>「満たしていない」チェックポイントがある場合、クラスタ順の優先リストが軸情報付きで表示されること</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Agile TPI</t>
+        </is>
+      </c>
+      <c r="F40" s="4" t="inlineStr">
+        <is>
+          <t>1. 一部チェックポイントを「満たしていない」にする
+2. 結果画面を開く</t>
+        </is>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>「改善優先度の高いチェックポイントは以下の通りです。」に続き、軸・キーエリア付きの優先リストが表示される</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="inlineStr"/>
+    </row>
+    <row r="41" ht="72" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>TC-40</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Agile TPI全達成メッセージ確認</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>全チェックポイントが「満たしている」の場合の固定メッセージ確認</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Agile TPI</t>
+        </is>
+      </c>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>1. 全項目を「満たしている」にする
+2. 結果画面を開く</t>
+        </is>
+      </c>
+      <c r="G41" s="4" t="inlineStr">
+        <is>
+          <t>「すべてのチェックポイントを満たしています。素晴らしい成果です！」が表示される</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>仕様に明記のなかったケースのため独自に追加</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="72" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>TC-41</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>優先チェックポイントの表記形式確認</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>「[クラスタ文字][キーエリア名]」（Agile TPIは軸名も含む）＋改行＋全角スペース1つ＋チェックポイント本文、の2行形式で出力されること</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>1. 短評出力内の優先チェックポイント項目を確認する</t>
+        </is>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>指定通りの改行・スペースを含む形式で出力される</t>
+        </is>
+      </c>
+      <c r="H42" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="inlineStr"/>
+    </row>
+    <row r="43" ht="72" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>TC-42</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>テキストエリアの編集可否確認</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>短評欄が編集可能なテキストエリアとして表示され、自由に加筆・修正できること</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>1. 短評テキストエリアの内容を書き換える</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>入力内容がそのまま反映される</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr"/>
+    </row>
+    <row r="44" ht="72" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>TC-43</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>回答未変更時の編集内容保持確認</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>短評を編集後、診断画面に戻り回答を一切変更せず結果画面へ戻った場合、編集内容がそのまま維持されること</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>1. 短評を編集する
+2. 診断画面へ移動する
+3. 変更せず「診断する」を押す
+4. 結果画面の短評を確認する</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>編集した内容がそのまま表示される</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>TPI NEXT・Agile TPI両方で確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="72" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>TC-44</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>回答変更時の短評再生成確認</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>短評編集後、診断画面で回答を1件変更して結果画面へ戻ると、編集内容が破棄され新しい診断結果に基づくデフォルト文言が出力されること</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="inlineStr">
+        <is>
+          <t>1. 短評を編集する
+2. 診断画面へ移動する
+3. チェックポイントを1件変更する
+4. 「診断する」を押す
+5. 結果画面の短評を確認する</t>
+        </is>
+      </c>
+      <c r="G45" s="4" t="inlineStr">
+        <is>
+          <t>編集内容ではなく、新しい回答内容に基づいたデフォルト文言が表示される</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>PASS（修正前は編集内容が誤って残り続けFAIL）</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>commitReview()が回答オブジェクトの参照をそのまま保存していたため、後から回答が変わってもスナップショット側も連動して変化し、常に「変更なし」と誤判定される不具合を発見。複製（スプレッド構文）を保存するよう修正。TPI NEXT・Agile TPI両方で確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="72" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>TC-45</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>短評機能</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>回答クリア時の短評スナップショット削除確認</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>「回答をクリアする」実行時、比較用に保存していた短評スナップショット（tpiAssessmentTool.review.v1）も削除されること</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="inlineStr">
+        <is>
+          <t>1. 短評を編集する
+2. 「回答をクリアする」を実行する
+3. localStorageを確認する</t>
+        </is>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>該当フレームワークの短評スナップショットが空になる</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>TPI NEXT・Agile TPI両方で確認</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="72" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>TC-46</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>非機能</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>JSランタイムエラーの非発生確認（フェーズ4以降）</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>マトリクス・スパイダーグラフ・メモ機能・回答クリア・短評機能のテストを通じて、ブラウザコンソールにエラーが出力されていないこと</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>共通</t>
+        </is>
+      </c>
+      <c r="F47" s="4" t="inlineStr">
+        <is>
+          <t>各テストケース実施後にブラウザの開発者コンソールのログを確認する</t>
+        </is>
+      </c>
+      <c r="G47" s="4" t="inlineStr">
+        <is>
+          <t>エラーログが出力されない</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>全テストケース実施を通じて継続的に確認</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J20"/>
+  <autoFilter ref="A1:J47"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>